<commit_message>
EN/DE translations live for hymns 1-40
merge-translations.mjs folds staging sheets into the live xlsx (spliceRows is a no-op in bundled exceljs, rewrites in place); drafts data moved to content/drafts/ so check-hymns ignores them; hymn 15 ellipsis completed; import 1000 Arabic + 40 EN + 40 DE, checks green; hymn 1 translations byte-identical.
</commit_message>
<xml_diff>
--- a/content/staging-en-de-001-020.xlsx
+++ b/content/staging-en-de-001-020.xlsx
@@ -1953,7 +1953,7 @@
     <t>That they may receive a portion too</t>
   </si>
   <si>
-    <t>As I received, shouting and saying…</t>
+    <t>As I received, shouting and proclaiming</t>
   </si>
   <si>
     <t>Trample On, O Soul, With Courage</t>
@@ -3024,7 +3024,7 @@
     <t>Dass auch sie Anteil empfangen</t>
   </si>
   <si>
-    <t>Wie ich empfing, rufend und sprechend…</t>
+    <t>Wie ich empfing, rufend und verkündend</t>
   </si>
   <si>
     <t>Zertritt, o Seele, mit Mut</t>

</xml_diff>